<commit_message>
fix(journey): remove lojas uniar, poloar e dufrio substituindo por frigelar, clima rio e havan
</commit_message>
<xml_diff>
--- a/public/Journey Novembro 2026 - Opcao 2.xlsx
+++ b/public/Journey Novembro 2026 - Opcao 2.xlsx
@@ -8100,7 +8100,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>S00170 - UNIAR - AVENIDA. AYRTON SENNA - 1.850 - RIO DE JANEIRO - RJ</t>
+          <t>S06150 - FRIGELAR - AVENIDA AYRTON SENNA - 4701 - RIO DE JANEIRO - RJ</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
@@ -8110,7 +8110,7 @@
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>UNIAR</t>
+          <t>FRIGELAR</t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
@@ -8125,7 +8125,7 @@
       </c>
       <c r="L91" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="M91" t="inlineStr">
@@ -8361,7 +8361,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>S00141 - UNIAR - RUA MARIZ E BARROS - 521 - NITEROI - RJ</t>
+          <t>S00164 - CLIMA RIO - RUA MANOEL JOAO GONCALVES - 84 - SAO GONCALO - RJ</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
@@ -8371,12 +8371,12 @@
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>UNIAR</t>
+          <t>CLIMA RIO</t>
         </is>
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>NITEROI</t>
+          <t>SAO GONCALO</t>
         </is>
       </c>
       <c r="K94" t="inlineStr">
@@ -8970,7 +8970,7 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>S00170 - UNIAR - AVENIDA. AYRTON SENNA - 1.850 - RIO DE JANEIRO - RJ</t>
+          <t>S06150 - FRIGELAR - AVENIDA AYRTON SENNA - 4701 - RIO DE JANEIRO - RJ</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
@@ -8980,7 +8980,7 @@
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>UNIAR</t>
+          <t>FRIGELAR</t>
         </is>
       </c>
       <c r="J101" t="inlineStr">
@@ -8995,7 +8995,7 @@
       </c>
       <c r="L101" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="M101" t="inlineStr">
@@ -9978,7 +9978,7 @@
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>S00141 - UNIAR - RUA MARIZ E BARROS - 521 - NITEROI - RJ</t>
+          <t>S00164 - CLIMA RIO - RUA MANOEL JOAO GONCALVES - 84 - SAO GONCALO - RJ</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
@@ -9988,12 +9988,12 @@
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>UNIAR</t>
+          <t>CLIMA RIO</t>
         </is>
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>NITEROI</t>
+          <t>SAO GONCALO</t>
         </is>
       </c>
       <c r="K113" t="inlineStr">
@@ -10413,7 +10413,7 @@
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>S00170 - UNIAR - AVENIDA. AYRTON SENNA - 1.850 - RIO DE JANEIRO - RJ</t>
+          <t>S06150 - FRIGELAR - AVENIDA AYRTON SENNA - 4701 - RIO DE JANEIRO - RJ</t>
         </is>
       </c>
       <c r="H118" t="inlineStr">
@@ -10423,7 +10423,7 @@
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>UNIAR</t>
+          <t>FRIGELAR</t>
         </is>
       </c>
       <c r="J118" t="inlineStr">
@@ -10438,7 +10438,7 @@
       </c>
       <c r="L118" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="M118" t="inlineStr">
@@ -11160,7 +11160,7 @@
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>S00148 - UNIAR - R. DOM PEDRO II - 390 - PORTO ALEGRE - RS</t>
+          <t>S01271 - FRIGELAR - AVENIDA PERNAMBUCO - 2273 - PORTO ALEGRE - RS</t>
         </is>
       </c>
       <c r="H127" t="inlineStr">
@@ -11170,7 +11170,7 @@
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>UNIAR</t>
+          <t>FRIGELAR</t>
         </is>
       </c>
       <c r="J127" t="inlineStr">
@@ -11185,7 +11185,7 @@
       </c>
       <c r="L127" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="M127" t="inlineStr">
@@ -11247,7 +11247,7 @@
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>S00229 - UNIAR - RUA PROFESSOR CRISTIANO FISCHER - 1400 - PORTO ALEGRE - RS</t>
+          <t>S00119 - FRIGELAR - AVENIDA PERNAMBUCO - 2285 - PORTO ALEGRE - RS</t>
         </is>
       </c>
       <c r="H128" t="inlineStr">
@@ -11257,7 +11257,7 @@
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>UNIAR</t>
+          <t>FRIGELAR</t>
         </is>
       </c>
       <c r="J128" t="inlineStr">
@@ -11272,7 +11272,7 @@
       </c>
       <c r="L128" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="M128" t="inlineStr">
@@ -12030,7 +12030,7 @@
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>S00148 - UNIAR - R. DOM PEDRO II - 390 - PORTO ALEGRE - RS</t>
+          <t>S15962 - HAVAN - RUA OTAVIO SCHEMES - 4105 - GRAVATAI - RS</t>
         </is>
       </c>
       <c r="H137" t="inlineStr">
@@ -12040,12 +12040,12 @@
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>UNIAR</t>
+          <t>HAVAN</t>
         </is>
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>PORTO ALEGRE</t>
+          <t>GRAVATAI</t>
         </is>
       </c>
       <c r="K137" t="inlineStr">
@@ -12055,7 +12055,7 @@
       </c>
       <c r="L137" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="M137" t="inlineStr">
@@ -12117,7 +12117,7 @@
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>S00229 - UNIAR - RUA PROFESSOR CRISTIANO FISCHER - 1400 - PORTO ALEGRE - RS</t>
+          <t>S18040 - HAVAN - AVENIDA ASSIS BRASIL - 11120 - PORTO ALEGRE - RS</t>
         </is>
       </c>
       <c r="H138" t="inlineStr">
@@ -12127,7 +12127,7 @@
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>UNIAR</t>
+          <t>HAVAN</t>
         </is>
       </c>
       <c r="J138" t="inlineStr">
@@ -12142,7 +12142,7 @@
       </c>
       <c r="L138" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="M138" t="inlineStr">
@@ -12900,7 +12900,7 @@
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>S00148 - UNIAR - R. DOM PEDRO II - 390 - PORTO ALEGRE - RS</t>
+          <t>S01271 - FRIGELAR - AVENIDA PERNAMBUCO - 2273 - PORTO ALEGRE - RS</t>
         </is>
       </c>
       <c r="H147" t="inlineStr">
@@ -12910,7 +12910,7 @@
       </c>
       <c r="I147" t="inlineStr">
         <is>
-          <t>UNIAR</t>
+          <t>FRIGELAR</t>
         </is>
       </c>
       <c r="J147" t="inlineStr">
@@ -12925,7 +12925,7 @@
       </c>
       <c r="L147" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="M147" t="inlineStr">
@@ -12987,7 +12987,7 @@
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>S00229 - UNIAR - RUA PROFESSOR CRISTIANO FISCHER - 1400 - PORTO ALEGRE - RS</t>
+          <t>S00119 - FRIGELAR - AVENIDA PERNAMBUCO - 2285 - PORTO ALEGRE - RS</t>
         </is>
       </c>
       <c r="H148" t="inlineStr">
@@ -12997,7 +12997,7 @@
       </c>
       <c r="I148" t="inlineStr">
         <is>
-          <t>UNIAR</t>
+          <t>FRIGELAR</t>
         </is>
       </c>
       <c r="J148" t="inlineStr">
@@ -13012,7 +13012,7 @@
       </c>
       <c r="L148" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="M148" t="inlineStr">
@@ -13647,7 +13647,7 @@
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t>S00148 - UNIAR - R. DOM PEDRO II - 390 - PORTO ALEGRE - RS</t>
+          <t>S15962 - HAVAN - RUA OTAVIO SCHEMES - 4105 - GRAVATAI - RS</t>
         </is>
       </c>
       <c r="H156" t="inlineStr">
@@ -13657,12 +13657,12 @@
       </c>
       <c r="I156" t="inlineStr">
         <is>
-          <t>UNIAR</t>
+          <t>HAVAN</t>
         </is>
       </c>
       <c r="J156" t="inlineStr">
         <is>
-          <t>PORTO ALEGRE</t>
+          <t>GRAVATAI</t>
         </is>
       </c>
       <c r="K156" t="inlineStr">
@@ -13672,7 +13672,7 @@
       </c>
       <c r="L156" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="M156" t="inlineStr">
@@ -13734,7 +13734,7 @@
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>S00229 - UNIAR - RUA PROFESSOR CRISTIANO FISCHER - 1400 - PORTO ALEGRE - RS</t>
+          <t>S18040 - HAVAN - AVENIDA ASSIS BRASIL - 11120 - PORTO ALEGRE - RS</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">
@@ -13744,7 +13744,7 @@
       </c>
       <c r="I157" t="inlineStr">
         <is>
-          <t>UNIAR</t>
+          <t>HAVAN</t>
         </is>
       </c>
       <c r="J157" t="inlineStr">
@@ -13759,7 +13759,7 @@
       </c>
       <c r="L157" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="M157" t="inlineStr">
@@ -14829,7 +14829,7 @@
       </c>
       <c r="G170" t="inlineStr">
         <is>
-          <t>S00901 - UNIAR - AV. DOUTOR CARLOS DE MORAES BARROS - 350 - OSASCO - SP</t>
+          <t>S06664 - FRIGELAR - AVENIDA PROF FRANCISCO MORATO - 3205 - SAO PAULO - SP</t>
         </is>
       </c>
       <c r="H170" t="inlineStr">
@@ -14839,12 +14839,12 @@
       </c>
       <c r="I170" t="inlineStr">
         <is>
-          <t>UNIAR</t>
+          <t>FRIGELAR</t>
         </is>
       </c>
       <c r="J170" t="inlineStr">
         <is>
-          <t>OSASCO</t>
+          <t>SAO PAULO</t>
         </is>
       </c>
       <c r="K170" t="inlineStr">
@@ -15090,7 +15090,7 @@
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t>S01983 - UNIAR - AVENIDA SUPLICY - 443 - GUARULHOS - SP</t>
+          <t>S04610 - FRIGELAR - AVENIDA MONTEIRO LOBATO - 393 - GUARULHOS - SP</t>
         </is>
       </c>
       <c r="H173" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="I173" t="inlineStr">
         <is>
-          <t>UNIAR</t>
+          <t>FRIGELAR</t>
         </is>
       </c>
       <c r="J173" t="inlineStr">
@@ -15264,7 +15264,7 @@
       </c>
       <c r="G175" t="inlineStr">
         <is>
-          <t>S00146 - UNIAR - RUA BARAO DE CAMPINAS - 690 - SAO PAULO - SP</t>
+          <t>S02324 - FRIGELAR - ALAMEDA GLETE - 908 - SAO PAULO - SP</t>
         </is>
       </c>
       <c r="H175" t="inlineStr">
@@ -15274,7 +15274,7 @@
       </c>
       <c r="I175" t="inlineStr">
         <is>
-          <t>UNIAR</t>
+          <t>FRIGELAR</t>
         </is>
       </c>
       <c r="J175" t="inlineStr">
@@ -15289,7 +15289,7 @@
       </c>
       <c r="L175" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="M175" t="inlineStr">
@@ -16707,7 +16707,7 @@
       </c>
       <c r="G192" t="inlineStr">
         <is>
-          <t>S01983 - UNIAR - AVENIDA SUPLICY - 443 - GUARULHOS - SP</t>
+          <t>S04610 - FRIGELAR - AVENIDA MONTEIRO LOBATO - 393 - GUARULHOS - SP</t>
         </is>
       </c>
       <c r="H192" t="inlineStr">
@@ -16717,7 +16717,7 @@
       </c>
       <c r="I192" t="inlineStr">
         <is>
-          <t>UNIAR</t>
+          <t>FRIGELAR</t>
         </is>
       </c>
       <c r="J192" t="inlineStr">
@@ -16881,7 +16881,7 @@
       </c>
       <c r="G194" t="inlineStr">
         <is>
-          <t>S00146 - UNIAR - RUA BARAO DE CAMPINAS - 690 - SAO PAULO - SP</t>
+          <t>S02324 - FRIGELAR - ALAMEDA GLETE - 908 - SAO PAULO - SP</t>
         </is>
       </c>
       <c r="H194" t="inlineStr">
@@ -16891,7 +16891,7 @@
       </c>
       <c r="I194" t="inlineStr">
         <is>
-          <t>UNIAR</t>
+          <t>FRIGELAR</t>
         </is>
       </c>
       <c r="J194" t="inlineStr">
@@ -16906,7 +16906,7 @@
       </c>
       <c r="L194" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="M194" t="inlineStr">
@@ -17316,7 +17316,7 @@
       </c>
       <c r="G199" t="inlineStr">
         <is>
-          <t>S00901 - UNIAR - AV. DOUTOR CARLOS DE MORAES BARROS - 350 - OSASCO - SP</t>
+          <t>S06664 - FRIGELAR - AVENIDA PROF FRANCISCO MORATO - 3205 - SAO PAULO - SP</t>
         </is>
       </c>
       <c r="H199" t="inlineStr">
@@ -17326,12 +17326,12 @@
       </c>
       <c r="I199" t="inlineStr">
         <is>
-          <t>UNIAR</t>
+          <t>FRIGELAR</t>
         </is>
       </c>
       <c r="J199" t="inlineStr">
         <is>
-          <t>OSASCO</t>
+          <t>SAO PAULO</t>
         </is>
       </c>
       <c r="K199" t="inlineStr">

</xml_diff>